<commit_message>
fixed streamflow rating curve
</commit_message>
<xml_diff>
--- a/data-dict.xlsx
+++ b/data-dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizacohn/Desktop/cascaded-hydro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB0BD7B-1748-D94B-B537-A6A17BB5C99F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536963A1-6F0A-DF45-882F-9776455D5526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="760" windowWidth="28740" windowHeight="17060" xr2:uid="{91E4E570-4FDA-D248-8E42-05C4D408F481}"/>
+    <workbookView xWindow="180" yWindow="760" windowWidth="28740" windowHeight="16920" xr2:uid="{91E4E570-4FDA-D248-8E42-05C4D408F481}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
convex hull approx begin;'
</commit_message>
<xml_diff>
--- a/data-dict.xlsx
+++ b/data-dict.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizacohn/Desktop/cascaded-hydro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA38CDD8-E3D0-A94B-B831-E9FE142537A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25880A4D-AD16-994A-861B-1A33D73DFE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="760" windowWidth="28740" windowHeight="16920" xr2:uid="{91E4E570-4FDA-D248-8E42-05C4D408F481}"/>
+    <workbookView xWindow="180" yWindow="760" windowWidth="28740" windowHeight="16920" activeTab="1" xr2:uid="{91E4E570-4FDA-D248-8E42-05C4D408F481}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>

</xml_diff>